<commit_message>
Update 49_53_66.xlsx to Dual Missing Data Protocol & Rule 19 layout, and document V5 architectural release in CHANGELOG.md
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/49_53_66.xlsx
+++ b/03_Coding_Sheets/49_53_66.xlsx
@@ -709,12 +709,14 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B4" t="n">
         <v>49</v>
       </c>
-      <c r="C4" t="n">
-        <v>49</v>
-      </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
@@ -728,6 +730,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>250</v>
+      </c>
+      <c r="W4" t="n">
+        <v>999</v>
+      </c>
+      <c r="X4" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>999</v>
+      </c>
       <c r="AA4" t="n">
         <v>4</v>
       </c>
@@ -737,11 +761,6 @@
       <c r="AC4" t="n">
         <v>999</v>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF4" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -756,11 +775,6 @@
       <c r="AJ4" t="n">
         <v>5</v>
       </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM4" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -804,12 +818,14 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B5" t="n">
         <v>49</v>
       </c>
-      <c r="C5" t="n">
-        <v>49</v>
-      </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
@@ -823,6 +839,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>250</v>
+      </c>
+      <c r="W5" t="n">
+        <v>999</v>
+      </c>
+      <c r="X5" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>999</v>
+      </c>
       <c r="AA5" t="n">
         <v>4</v>
       </c>
@@ -832,11 +870,6 @@
       <c r="AC5" t="n">
         <v>999</v>
       </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF5" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -851,11 +884,6 @@
       <c r="AJ5" t="n">
         <v>5</v>
       </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM5" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -899,12 +927,14 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B6" t="n">
         <v>49</v>
       </c>
-      <c r="C6" t="n">
-        <v>49</v>
-      </c>
       <c r="D6" t="n">
         <v>3</v>
       </c>
@@ -918,6 +948,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>250</v>
+      </c>
+      <c r="W6" t="n">
+        <v>999</v>
+      </c>
+      <c r="X6" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>999</v>
+      </c>
       <c r="AA6" t="n">
         <v>4</v>
       </c>
@@ -927,11 +979,6 @@
       <c r="AC6" t="n">
         <v>999</v>
       </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF6" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -946,11 +993,6 @@
       <c r="AJ6" t="n">
         <v>5</v>
       </c>
-      <c r="AK6" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM6" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -994,12 +1036,14 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B7" t="n">
         <v>49</v>
       </c>
-      <c r="C7" t="n">
-        <v>49</v>
-      </c>
       <c r="D7" t="n">
         <v>4</v>
       </c>
@@ -1013,6 +1057,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>250</v>
+      </c>
+      <c r="W7" t="n">
+        <v>999</v>
+      </c>
+      <c r="X7" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>999</v>
+      </c>
       <c r="AA7" t="n">
         <v>4</v>
       </c>
@@ -1022,11 +1088,6 @@
       <c r="AC7" t="n">
         <v>999</v>
       </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF7" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1041,11 +1102,6 @@
       <c r="AJ7" t="n">
         <v>5</v>
       </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM7" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1089,12 +1145,14 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B8" t="n">
         <v>49</v>
       </c>
-      <c r="C8" t="n">
-        <v>49</v>
-      </c>
       <c r="D8" t="n">
         <v>5</v>
       </c>
@@ -1108,6 +1166,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>250</v>
+      </c>
+      <c r="W8" t="n">
+        <v>999</v>
+      </c>
+      <c r="X8" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>999</v>
+      </c>
       <c r="AA8" t="n">
         <v>4</v>
       </c>
@@ -1117,11 +1197,6 @@
       <c r="AC8" t="n">
         <v>999</v>
       </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF8" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1136,11 +1211,6 @@
       <c r="AJ8" t="n">
         <v>5</v>
       </c>
-      <c r="AK8" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM8" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1184,12 +1254,14 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B9" t="n">
         <v>49</v>
       </c>
-      <c r="C9" t="n">
-        <v>49</v>
-      </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
@@ -1203,6 +1275,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>250</v>
+      </c>
+      <c r="W9" t="n">
+        <v>999</v>
+      </c>
+      <c r="X9" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>999</v>
+      </c>
       <c r="AA9" t="n">
         <v>4</v>
       </c>
@@ -1212,11 +1306,6 @@
       <c r="AC9" t="n">
         <v>999</v>
       </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF9" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1231,11 +1320,6 @@
       <c r="AJ9" t="n">
         <v>5</v>
       </c>
-      <c r="AK9" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM9" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1279,12 +1363,14 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B10" t="n">
         <v>49</v>
       </c>
-      <c r="C10" t="n">
-        <v>49</v>
-      </c>
       <c r="D10" t="n">
         <v>7</v>
       </c>
@@ -1298,6 +1384,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>250</v>
+      </c>
+      <c r="W10" t="n">
+        <v>999</v>
+      </c>
+      <c r="X10" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>999</v>
+      </c>
       <c r="AA10" t="n">
         <v>4</v>
       </c>
@@ -1307,11 +1415,6 @@
       <c r="AC10" t="n">
         <v>999</v>
       </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF10" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1326,11 +1429,6 @@
       <c r="AJ10" t="n">
         <v>5</v>
       </c>
-      <c r="AK10" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM10" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1374,12 +1472,14 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B11" t="n">
         <v>49</v>
       </c>
-      <c r="C11" t="n">
-        <v>49</v>
-      </c>
       <c r="D11" t="n">
         <v>8</v>
       </c>
@@ -1393,6 +1493,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>250</v>
+      </c>
+      <c r="W11" t="n">
+        <v>999</v>
+      </c>
+      <c r="X11" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>999</v>
+      </c>
       <c r="AA11" t="n">
         <v>4</v>
       </c>
@@ -1402,11 +1524,6 @@
       <c r="AC11" t="n">
         <v>999</v>
       </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF11" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1421,11 +1538,6 @@
       <c r="AJ11" t="n">
         <v>5</v>
       </c>
-      <c r="AK11" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM11" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1469,12 +1581,14 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B12" t="n">
         <v>49</v>
       </c>
-      <c r="C12" t="n">
-        <v>49</v>
-      </c>
       <c r="D12" t="n">
         <v>9</v>
       </c>
@@ -1488,6 +1602,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>250</v>
+      </c>
+      <c r="W12" t="n">
+        <v>999</v>
+      </c>
+      <c r="X12" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>999</v>
+      </c>
       <c r="AA12" t="n">
         <v>4</v>
       </c>
@@ -1497,11 +1633,6 @@
       <c r="AC12" t="n">
         <v>999</v>
       </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF12" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1516,11 +1647,6 @@
       <c r="AJ12" t="n">
         <v>5</v>
       </c>
-      <c r="AK12" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM12" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1564,12 +1690,14 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B13" t="n">
         <v>49</v>
       </c>
-      <c r="C13" t="n">
-        <v>49</v>
-      </c>
       <c r="D13" t="n">
         <v>10</v>
       </c>
@@ -1583,6 +1711,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>250</v>
+      </c>
+      <c r="W13" t="n">
+        <v>999</v>
+      </c>
+      <c r="X13" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>999</v>
+      </c>
       <c r="AA13" t="n">
         <v>4</v>
       </c>
@@ -1592,11 +1742,6 @@
       <c r="AC13" t="n">
         <v>999</v>
       </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF13" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1611,11 +1756,6 @@
       <c r="AJ13" t="n">
         <v>5</v>
       </c>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM13" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1659,12 +1799,14 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B14" t="n">
         <v>49</v>
       </c>
-      <c r="C14" t="n">
-        <v>49</v>
-      </c>
       <c r="D14" t="n">
         <v>11</v>
       </c>
@@ -1678,6 +1820,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>250</v>
+      </c>
+      <c r="W14" t="n">
+        <v>999</v>
+      </c>
+      <c r="X14" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>999</v>
+      </c>
       <c r="AA14" t="n">
         <v>5</v>
       </c>
@@ -1687,11 +1851,6 @@
       <c r="AC14" t="n">
         <v>999</v>
       </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF14" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1706,11 +1865,6 @@
       <c r="AJ14" t="n">
         <v>5</v>
       </c>
-      <c r="AK14" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM14" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1754,12 +1908,14 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B15" t="n">
         <v>49</v>
       </c>
-      <c r="C15" t="n">
-        <v>49</v>
-      </c>
       <c r="D15" t="n">
         <v>12</v>
       </c>
@@ -1773,6 +1929,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>250</v>
+      </c>
+      <c r="W15" t="n">
+        <v>999</v>
+      </c>
+      <c r="X15" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>999</v>
+      </c>
       <c r="AA15" t="n">
         <v>5</v>
       </c>
@@ -1782,11 +1960,6 @@
       <c r="AC15" t="n">
         <v>999</v>
       </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF15" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1801,11 +1974,6 @@
       <c r="AJ15" t="n">
         <v>5</v>
       </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM15" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1849,12 +2017,14 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B16" t="n">
         <v>49</v>
       </c>
-      <c r="C16" t="n">
-        <v>49</v>
-      </c>
       <c r="D16" t="n">
         <v>13</v>
       </c>
@@ -1868,6 +2038,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>250</v>
+      </c>
+      <c r="W16" t="n">
+        <v>999</v>
+      </c>
+      <c r="X16" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>999</v>
+      </c>
       <c r="AA16" t="n">
         <v>5</v>
       </c>
@@ -1877,11 +2069,6 @@
       <c r="AC16" t="n">
         <v>999</v>
       </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF16" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1896,11 +2083,6 @@
       <c r="AJ16" t="n">
         <v>5</v>
       </c>
-      <c r="AK16" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM16" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -1944,12 +2126,14 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B17" t="n">
         <v>49</v>
       </c>
-      <c r="C17" t="n">
-        <v>49</v>
-      </c>
       <c r="D17" t="n">
         <v>14</v>
       </c>
@@ -1963,6 +2147,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>250</v>
+      </c>
+      <c r="W17" t="n">
+        <v>999</v>
+      </c>
+      <c r="X17" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>999</v>
+      </c>
       <c r="AA17" t="n">
         <v>5</v>
       </c>
@@ -1972,11 +2178,6 @@
       <c r="AC17" t="n">
         <v>999</v>
       </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF17" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -1991,11 +2192,6 @@
       <c r="AJ17" t="n">
         <v>5</v>
       </c>
-      <c r="AK17" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM17" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -2039,12 +2235,14 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B18" t="n">
         <v>49</v>
       </c>
-      <c r="C18" t="n">
-        <v>49</v>
-      </c>
       <c r="D18" t="n">
         <v>15</v>
       </c>
@@ -2058,6 +2256,28 @@
           <t>2 = Longitudinal design</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>250</v>
+      </c>
+      <c r="W18" t="n">
+        <v>999</v>
+      </c>
+      <c r="X18" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>999</v>
+      </c>
       <c r="AA18" t="n">
         <v>5</v>
       </c>
@@ -2067,11 +2287,6 @@
       <c r="AC18" t="n">
         <v>999</v>
       </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF18" t="inlineStr">
         <is>
           <t>COBSBs</t>
@@ -2086,11 +2301,6 @@
       <c r="AJ18" t="n">
         <v>5</v>
       </c>
-      <c r="AK18" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM18" t="inlineStr">
         <is>
           <t>spiritual leadership scale</t>
@@ -2134,12 +2344,14 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B19" t="n">
         <v>53</v>
       </c>
-      <c r="C19" t="n">
-        <v>53</v>
-      </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
@@ -2156,6 +2368,15 @@
       <c r="V19" t="n">
         <v>1461</v>
       </c>
+      <c r="W19" t="n">
+        <v>999</v>
+      </c>
+      <c r="X19" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>999</v>
+      </c>
       <c r="AA19" t="n">
         <v>2</v>
       </c>
@@ -2165,11 +2386,6 @@
       <c r="AC19" t="n">
         <v>5</v>
       </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF19" t="inlineStr">
         <is>
           <t>identification with the branch</t>
@@ -2184,11 +2400,6 @@
       <c r="AJ19" t="n">
         <v>7</v>
       </c>
-      <c r="AK19" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM19" t="inlineStr">
         <is>
           <t>locus of control scale</t>
@@ -2227,12 +2438,14 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B20" t="n">
         <v>53</v>
       </c>
-      <c r="C20" t="n">
-        <v>53</v>
-      </c>
       <c r="D20" t="n">
         <v>2</v>
       </c>
@@ -2249,6 +2462,15 @@
       <c r="V20" t="n">
         <v>1461</v>
       </c>
+      <c r="W20" t="n">
+        <v>999</v>
+      </c>
+      <c r="X20" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>999</v>
+      </c>
       <c r="AA20" t="n">
         <v>2</v>
       </c>
@@ -2258,11 +2480,6 @@
       <c r="AC20" t="n">
         <v>5</v>
       </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF20" t="inlineStr">
         <is>
           <t>identification with the branch</t>
@@ -2277,11 +2494,6 @@
       <c r="AJ20" t="n">
         <v>7</v>
       </c>
-      <c r="AK20" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM20" t="inlineStr">
         <is>
           <t>performance control</t>
@@ -2320,12 +2532,14 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B21" t="n">
         <v>53</v>
       </c>
-      <c r="C21" t="n">
-        <v>53</v>
-      </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
@@ -2342,6 +2556,15 @@
       <c r="V21" t="n">
         <v>1461</v>
       </c>
+      <c r="W21" t="n">
+        <v>999</v>
+      </c>
+      <c r="X21" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>999</v>
+      </c>
       <c r="AA21" t="n">
         <v>2</v>
       </c>
@@ -2351,11 +2574,6 @@
       <c r="AC21" t="n">
         <v>5</v>
       </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF21" t="inlineStr">
         <is>
           <t>identification with the branch</t>
@@ -2370,11 +2588,6 @@
       <c r="AJ21" t="n">
         <v>100</v>
       </c>
-      <c r="AK21" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM21" t="inlineStr">
         <is>
           <t>TRI*M index</t>
@@ -2413,12 +2626,14 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B22" t="n">
         <v>53</v>
       </c>
-      <c r="C22" t="n">
-        <v>53</v>
-      </c>
       <c r="D22" t="n">
         <v>4</v>
       </c>
@@ -2435,6 +2650,15 @@
       <c r="V22" t="n">
         <v>1461</v>
       </c>
+      <c r="W22" t="n">
+        <v>999</v>
+      </c>
+      <c r="X22" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>999</v>
+      </c>
       <c r="AA22" t="n">
         <v>2</v>
       </c>
@@ -2444,11 +2668,6 @@
       <c r="AC22" t="n">
         <v>6</v>
       </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF22" t="inlineStr">
         <is>
           <t>CS-related meetings between managers and colleagues</t>
@@ -2463,11 +2682,6 @@
       <c r="AJ22" t="n">
         <v>7</v>
       </c>
-      <c r="AK22" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM22" t="inlineStr">
         <is>
           <t>locus of control scale</t>
@@ -2506,12 +2720,14 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B23" t="n">
         <v>53</v>
       </c>
-      <c r="C23" t="n">
-        <v>53</v>
-      </c>
       <c r="D23" t="n">
         <v>5</v>
       </c>
@@ -2528,6 +2744,15 @@
       <c r="V23" t="n">
         <v>1461</v>
       </c>
+      <c r="W23" t="n">
+        <v>999</v>
+      </c>
+      <c r="X23" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>999</v>
+      </c>
       <c r="AA23" t="n">
         <v>2</v>
       </c>
@@ -2537,11 +2762,6 @@
       <c r="AC23" t="n">
         <v>6</v>
       </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF23" t="inlineStr">
         <is>
           <t>CS-related meetings between managers and colleagues</t>
@@ -2556,11 +2776,6 @@
       <c r="AJ23" t="n">
         <v>7</v>
       </c>
-      <c r="AK23" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM23" t="inlineStr">
         <is>
           <t>performance control</t>
@@ -2599,12 +2814,14 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B24" t="n">
         <v>53</v>
       </c>
-      <c r="C24" t="n">
-        <v>53</v>
-      </c>
       <c r="D24" t="n">
         <v>6</v>
       </c>
@@ -2621,6 +2838,15 @@
       <c r="V24" t="n">
         <v>1461</v>
       </c>
+      <c r="W24" t="n">
+        <v>999</v>
+      </c>
+      <c r="X24" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>999</v>
+      </c>
       <c r="AA24" t="n">
         <v>2</v>
       </c>
@@ -2630,11 +2856,6 @@
       <c r="AC24" t="n">
         <v>6</v>
       </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AF24" t="inlineStr">
         <is>
           <t>CS-related meetings between managers and colleagues</t>
@@ -2649,11 +2870,6 @@
       <c r="AJ24" t="n">
         <v>100</v>
       </c>
-      <c r="AK24" t="inlineStr">
-        <is>
-          <t>Not Reported</t>
-        </is>
-      </c>
       <c r="AM24" t="inlineStr">
         <is>
           <t>TRI*M index</t>
@@ -2692,12 +2908,14 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
       <c r="B25" t="n">
         <v>66</v>
       </c>
-      <c r="C25" t="n">
-        <v>66</v>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>0 = exclude</t>
@@ -2705,12 +2923,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Level of Analysis</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>[Level of Analysis violation]. Verbatim Evidence: "[Methodology] Project leaders were required to complete the questionnaire with reference to a completed NPD project." "[Abstract] A Partial Least Squares test on 73 NPD projects showed that..."</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Institutionalize Effect Size Provenance Protocol: enforce Table (p. Y) coordinate prefix and mandatory verbatim quote evidence for methodological flags in Col 50
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/49_53_66.xlsx
+++ b/03_Coding_Sheets/49_53_66.xlsx
@@ -813,7 +813,7 @@
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Vision, Col: External Representation, Raw: 0.314 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Hope/Faith, Col: External Representation, Raw: 0.318 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Altruistic love, Col: External Representation, Raw: 0.36 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Calling, Col: External Representation, Raw: 0.526 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Member, Col: External Representation, Raw: 0.535 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Vision, Col: Internalized Influence, Raw: 0.254 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Hope/Faith, Col: Internalized Influence, Raw: 0.289 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Altruistic love, Col: Internalized Influence, Raw: 0.313 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Calling, Col: Internalized Influence, Raw: 0.505 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Member, Col: Internalized Influence, Raw: 0.505 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Vision, Col: Service Delivery, Raw: 0.28 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="AX15" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Hope/Faith, Col: Service Delivery, Raw: 0.392 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="AX16" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Altruistic love, Col: Service Delivery, Raw: 0.371 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Calling, Col: Service Delivery, Raw: 0.479 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="AX18" t="inlineStr">
         <is>
-          <t>Based on latent variables</t>
+          <t>Table 2 (p. 556), Row: Member, Col: Service Delivery, Raw: 0.491 | Latent correlation: [Table 2 Note] "Figures on the diagonal represent the AVEs square roots."</t>
         </is>
       </c>
     </row>
@@ -2436,6 +2436,11 @@
       <c r="AW19" t="n">
         <v>-0.01</v>
       </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: Locus of control, Col: Branch identification, Raw: -0.01</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2530,6 +2535,11 @@
       <c r="AW20" t="n">
         <v>0.26</v>
       </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: Performance control, Col: Branch identification, Raw: 0.26</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2624,6 +2634,11 @@
       <c r="AW21" t="n">
         <v>0.06</v>
       </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: CS, Col: Branch identification, Raw: 0.06</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2718,6 +2733,11 @@
       <c r="AW22" t="n">
         <v>-0.02</v>
       </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: Locus of control, Col: CS-related meetings, Raw: -0.02</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2812,6 +2832,11 @@
       <c r="AW23" t="n">
         <v>0.1</v>
       </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: Performance control, Col: CS-related meetings, Raw: 0.1</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2905,6 +2930,11 @@
       </c>
       <c r="AW24" t="n">
         <v>0.02</v>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 671), Row: CS, Col: CS-related meetings, Raw: 0.02</t>
+        </is>
       </c>
     </row>
     <row r="25">

</xml_diff>